<commit_message>
feat(resources): add literature review templates
</commit_message>
<xml_diff>
--- a/templates/concept-context-grid.xlsx
+++ b/templates/concept-context-grid.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concept Grid" sheetId="1" r:id="R4f0334abc7f844ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rd7b3f92d38be4b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Concept Grid" sheetId="1" r:id="Ra819ca7415aa4211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rb0e218a8833a477b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -176,7 +176,7 @@
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -693,7 +693,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>0.1 discussion draft, 2026-07-12</x:v>
+        <x:v>0.2 discussion draft, 2026-07-13</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>